<commit_message>
new GST notification Circular notification
</commit_message>
<xml_diff>
--- a/backend/PDF_DOC/GST/Circulars/Circulars - CGST/Circulars - CGST.xlsx
+++ b/backend/PDF_DOC/GST/Circulars/Circulars - CGST/Circulars - CGST.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{250D8303-F4DA-40A5-A9F2-FAF885884AF3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB11BE47-0838-423F-88D9-E28CEFEA251E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="2026" sheetId="1" r:id="rId1"/>
+    <sheet name="2026" sheetId="4" r:id="rId1"/>
     <sheet name="2025" sheetId="2" r:id="rId2"/>
     <sheet name="2024" sheetId="3" r:id="rId3"/>
   </sheets>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="106">
   <si>
     <t>Circulars - CGST : 2024</t>
   </si>
@@ -328,6 +328,18 @@
   </si>
   <si>
     <t>Regularizing payment of GST on co-insurance premium apportioned by the lead insurer to the co-insurer and on ceding /re-insurance commission deducted from the reinsurance premium paid by the insurer to the reinsurer.</t>
+  </si>
+  <si>
+    <t>255/01/2026-GST</t>
+  </si>
+  <si>
+    <t>Clarification regarding jurisdiction in cases involving migration/ transfer of taxable persons from one jurisdiction to another jurisdiction</t>
+  </si>
+  <si>
+    <t>256/02/2026-GST</t>
+  </si>
+  <si>
+    <t>Clariﬁcation regarding ﬁling of appeal by department before the Goods and Services Appellate Tribunal against order of appellate authority (where Orders-in-Original have been passed by a Common Adjudicating Authority in DGGI cases).</t>
   </si>
 </sst>
 </file>
@@ -359,12 +371,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -379,7 +397,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -388,6 +406,11 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="15" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -669,10 +692,90 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A6A5DAD-A2D3-4A27-BB76-8CA7296A0958}">
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
+    <col min="3" max="3" width="147.85546875" style="4" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B6" s="3"/>
+    </row>
+    <row r="7" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B7" s="7">
+        <v>46228</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B8" s="3"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>102</v>
+      </c>
+      <c r="B9" s="3">
+        <v>46198</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B10" s="3"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B12" s="3"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B14" s="3"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B16" s="3"/>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B18" s="3"/>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B20" s="3"/>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B22" s="3"/>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B24" s="3"/>
+    </row>
+    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B26" s="3"/>
+    </row>
+    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B28" s="3"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1053,7 +1156,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>39</v>
       </c>
@@ -1064,7 +1167,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>41</v>
       </c>
@@ -1075,7 +1178,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>43</v>
       </c>
@@ -1097,7 +1200,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>47</v>
       </c>
@@ -1130,7 +1233,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>53</v>
       </c>
@@ -1141,7 +1244,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>55</v>
       </c>
@@ -1152,7 +1255,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>57</v>
       </c>
@@ -1207,7 +1310,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="70" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>67</v>
       </c>
@@ -1240,7 +1343,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="76" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>73</v>
       </c>
@@ -1262,7 +1365,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="80" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>77</v>
       </c>

</xml_diff>